<commit_message>
Restrictions: gedeelde-middelen constraints per ronde
</commit_message>
<xml_diff>
--- a/SchandomInput.xlsx
+++ b/SchandomInput.xlsx
@@ -8,23 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Schandom 2027\NK-Schandom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68D9D4A8-E99B-4616-80E6-92BE1FB2CDFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B08FE8CA-73A7-414D-AAAF-66312C829785}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" tabRatio="867" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" tabRatio="867" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Players" sheetId="1" r:id="rId1"/>
-    <sheet name="Games" sheetId="2" r:id="rId2"/>
-    <sheet name="PrefsTWB" sheetId="3" r:id="rId3"/>
-    <sheet name="PrefsJAS" sheetId="7" r:id="rId4"/>
-    <sheet name="PrefsWOS" sheetId="8" r:id="rId5"/>
-    <sheet name="PrefsROS" sheetId="9" r:id="rId6"/>
-    <sheet name="PrefsMIS" sheetId="10" r:id="rId7"/>
-    <sheet name="PrefsBRB" sheetId="11" r:id="rId8"/>
-    <sheet name="PrefsLOK" sheetId="12" r:id="rId9"/>
-    <sheet name="Berger12" sheetId="4" r:id="rId10"/>
-    <sheet name="Berger10" sheetId="5" r:id="rId11"/>
-    <sheet name="Berger8" sheetId="6" r:id="rId12"/>
+    <sheet name="Restrictions" sheetId="13" r:id="rId2"/>
+    <sheet name="Games" sheetId="2" r:id="rId3"/>
+    <sheet name="PrefsTWB" sheetId="3" r:id="rId4"/>
+    <sheet name="PrefsJAS" sheetId="7" r:id="rId5"/>
+    <sheet name="PrefsWOS" sheetId="8" r:id="rId6"/>
+    <sheet name="PrefsROS" sheetId="9" r:id="rId7"/>
+    <sheet name="PrefsMIS" sheetId="10" r:id="rId8"/>
+    <sheet name="PrefsBRB" sheetId="11" r:id="rId9"/>
+    <sheet name="PrefsLOK" sheetId="12" r:id="rId10"/>
+    <sheet name="Berger12" sheetId="4" r:id="rId11"/>
+    <sheet name="Berger10" sheetId="5" r:id="rId12"/>
+    <sheet name="Berger8" sheetId="6" r:id="rId13"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="114">
   <si>
     <t>ID</t>
   </si>
@@ -98,9 +99,6 @@
     <t>Fischer Random</t>
   </si>
   <si>
-    <t>Horde Chess</t>
-  </si>
-  <si>
     <t>Jeu de Boule</t>
   </si>
   <si>
@@ -113,9 +111,6 @@
     <t>Memory</t>
   </si>
   <si>
-    <t>Pinguin</t>
-  </si>
-  <si>
     <t>Poker Texas Hold'em</t>
   </si>
   <si>
@@ -372,6 +367,24 @@
   </si>
   <si>
     <t>4:8</t>
+  </si>
+  <si>
+    <t>Max</t>
+  </si>
+  <si>
+    <t>gobord</t>
+  </si>
+  <si>
+    <t>schaken</t>
+  </si>
+  <si>
+    <t>Game</t>
+  </si>
+  <si>
+    <t>Go Moku</t>
+  </si>
+  <si>
+    <t>Pente</t>
   </si>
 </sst>
 </file>
@@ -786,7 +799,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B2" s="1">
         <v>2040</v>
@@ -842,7 +855,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B9" s="1">
         <v>2000</v>
@@ -855,228 +868,837 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4F6C5ED-CE4B-4A90-947D-21DA231DC860}">
+  <dimension ref="A1:G26"/>
+  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="19.73046875" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="16384" width="9.1328125" style="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="B1" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="6">
+        <v>13</v>
+      </c>
+      <c r="C2" s="6">
+        <v>13</v>
+      </c>
+      <c r="D2" s="6">
+        <v>13</v>
+      </c>
+      <c r="E2" s="6">
+        <v>13</v>
+      </c>
+      <c r="F2" s="6">
+        <v>13</v>
+      </c>
+      <c r="G2" s="6">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="6">
+        <v>16</v>
+      </c>
+      <c r="C3" s="6">
+        <v>16</v>
+      </c>
+      <c r="D3" s="6">
+        <v>16</v>
+      </c>
+      <c r="E3" s="6">
+        <v>16</v>
+      </c>
+      <c r="F3" s="6">
+        <v>16</v>
+      </c>
+      <c r="G3" s="6">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="6">
+        <v>12</v>
+      </c>
+      <c r="C4" s="6">
+        <v>12</v>
+      </c>
+      <c r="D4" s="6">
+        <v>12</v>
+      </c>
+      <c r="E4" s="6">
+        <v>12</v>
+      </c>
+      <c r="F4" s="6">
+        <v>12</v>
+      </c>
+      <c r="G4" s="6">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="6">
+        <v>8</v>
+      </c>
+      <c r="C5" s="6">
+        <v>8</v>
+      </c>
+      <c r="D5" s="6">
+        <v>8</v>
+      </c>
+      <c r="E5" s="6">
+        <v>8</v>
+      </c>
+      <c r="F5" s="6">
+        <v>8</v>
+      </c>
+      <c r="G5" s="6">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="6">
+        <v>5</v>
+      </c>
+      <c r="C6" s="6">
+        <v>5</v>
+      </c>
+      <c r="D6" s="6">
+        <v>5</v>
+      </c>
+      <c r="E6" s="6">
+        <v>5</v>
+      </c>
+      <c r="F6" s="6">
+        <v>5</v>
+      </c>
+      <c r="G6" s="6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="6">
+        <v>2</v>
+      </c>
+      <c r="C7" s="6">
+        <v>2</v>
+      </c>
+      <c r="D7" s="6">
+        <v>2</v>
+      </c>
+      <c r="E7" s="6">
+        <v>2</v>
+      </c>
+      <c r="F7" s="6">
+        <v>2</v>
+      </c>
+      <c r="G7" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="6">
+        <v>3</v>
+      </c>
+      <c r="C8" s="6">
+        <v>3</v>
+      </c>
+      <c r="D8" s="6">
+        <v>3</v>
+      </c>
+      <c r="E8" s="6">
+        <v>3</v>
+      </c>
+      <c r="F8" s="6">
+        <v>3</v>
+      </c>
+      <c r="G8" s="6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="6">
+        <v>9</v>
+      </c>
+      <c r="C9" s="6">
+        <v>9</v>
+      </c>
+      <c r="D9" s="6">
+        <v>9</v>
+      </c>
+      <c r="E9" s="6">
+        <v>9</v>
+      </c>
+      <c r="F9" s="6">
+        <v>9</v>
+      </c>
+      <c r="G9" s="6">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="6">
+        <v>27</v>
+      </c>
+      <c r="C10" s="6">
+        <v>27</v>
+      </c>
+      <c r="D10" s="6">
+        <v>27</v>
+      </c>
+      <c r="E10" s="6">
+        <v>27</v>
+      </c>
+      <c r="F10" s="6">
+        <v>27</v>
+      </c>
+      <c r="G10" s="6">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="6">
+        <v>17</v>
+      </c>
+      <c r="C11" s="6">
+        <v>17</v>
+      </c>
+      <c r="D11" s="6">
+        <v>17</v>
+      </c>
+      <c r="E11" s="6">
+        <v>17</v>
+      </c>
+      <c r="F11" s="6">
+        <v>17</v>
+      </c>
+      <c r="G11" s="6">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>112</v>
+      </c>
+      <c r="B12" s="6">
+        <v>23</v>
+      </c>
+      <c r="C12" s="6">
+        <v>23</v>
+      </c>
+      <c r="D12" s="6">
+        <v>23</v>
+      </c>
+      <c r="E12" s="6">
+        <v>23</v>
+      </c>
+      <c r="F12" s="6">
+        <v>23</v>
+      </c>
+      <c r="G12" s="6">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13" s="6">
+        <v>15</v>
+      </c>
+      <c r="C13" s="6">
+        <v>15</v>
+      </c>
+      <c r="D13" s="6">
+        <v>15</v>
+      </c>
+      <c r="E13" s="6">
+        <v>15</v>
+      </c>
+      <c r="F13" s="6">
+        <v>15</v>
+      </c>
+      <c r="G13" s="6">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" s="6">
+        <v>0</v>
+      </c>
+      <c r="C14" s="6">
+        <v>0</v>
+      </c>
+      <c r="D14" s="6">
+        <v>0</v>
+      </c>
+      <c r="E14" s="6">
+        <v>0</v>
+      </c>
+      <c r="F14" s="6">
+        <v>0</v>
+      </c>
+      <c r="G14" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" s="6">
+        <v>28</v>
+      </c>
+      <c r="C15" s="6">
+        <v>28</v>
+      </c>
+      <c r="D15" s="6">
+        <v>28</v>
+      </c>
+      <c r="E15" s="6">
+        <v>28</v>
+      </c>
+      <c r="F15" s="6">
+        <v>28</v>
+      </c>
+      <c r="G15" s="6">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" s="6">
+        <v>14</v>
+      </c>
+      <c r="C16" s="6">
+        <v>14</v>
+      </c>
+      <c r="D16" s="6">
+        <v>14</v>
+      </c>
+      <c r="E16" s="6">
+        <v>14</v>
+      </c>
+      <c r="F16" s="6">
+        <v>14</v>
+      </c>
+      <c r="G16" s="6">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A17" t="s">
+        <v>113</v>
+      </c>
+      <c r="B17" s="6">
+        <v>24</v>
+      </c>
+      <c r="C17" s="6">
+        <v>24</v>
+      </c>
+      <c r="D17" s="6">
+        <v>24</v>
+      </c>
+      <c r="E17" s="6">
+        <v>24</v>
+      </c>
+      <c r="F17" s="6">
+        <v>24</v>
+      </c>
+      <c r="G17" s="6">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A18" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" s="6">
+        <v>0</v>
+      </c>
+      <c r="C18" s="6">
+        <v>0</v>
+      </c>
+      <c r="D18" s="6">
+        <v>0</v>
+      </c>
+      <c r="E18" s="6">
+        <v>0</v>
+      </c>
+      <c r="F18" s="6">
+        <v>0</v>
+      </c>
+      <c r="G18" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A19" t="s">
+        <v>23</v>
+      </c>
+      <c r="B19" s="6">
+        <v>0</v>
+      </c>
+      <c r="C19" s="6">
+        <v>0</v>
+      </c>
+      <c r="D19" s="6">
+        <v>0</v>
+      </c>
+      <c r="E19" s="6">
+        <v>0</v>
+      </c>
+      <c r="F19" s="6">
+        <v>0</v>
+      </c>
+      <c r="G19" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A20" t="s">
+        <v>24</v>
+      </c>
+      <c r="B20" s="6">
+        <v>6</v>
+      </c>
+      <c r="C20" s="6">
+        <v>6</v>
+      </c>
+      <c r="D20" s="6">
+        <v>6</v>
+      </c>
+      <c r="E20" s="6">
+        <v>6</v>
+      </c>
+      <c r="F20" s="6">
+        <v>6</v>
+      </c>
+      <c r="G20" s="6">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A21" t="s">
+        <v>25</v>
+      </c>
+      <c r="B21" s="6">
+        <v>19</v>
+      </c>
+      <c r="C21" s="6">
+        <v>19</v>
+      </c>
+      <c r="D21" s="6">
+        <v>19</v>
+      </c>
+      <c r="E21" s="6">
+        <v>19</v>
+      </c>
+      <c r="F21" s="6">
+        <v>19</v>
+      </c>
+      <c r="G21" s="6">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A22" t="s">
+        <v>26</v>
+      </c>
+      <c r="B22" s="6">
+        <v>25</v>
+      </c>
+      <c r="C22" s="6">
+        <v>25</v>
+      </c>
+      <c r="D22" s="6">
+        <v>25</v>
+      </c>
+      <c r="E22" s="6">
+        <v>25</v>
+      </c>
+      <c r="F22" s="6">
+        <v>25</v>
+      </c>
+      <c r="G22" s="6">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A23" t="s">
+        <v>27</v>
+      </c>
+      <c r="B23" s="6">
+        <v>18</v>
+      </c>
+      <c r="C23" s="6">
+        <v>18</v>
+      </c>
+      <c r="D23" s="6">
+        <v>18</v>
+      </c>
+      <c r="E23" s="6">
+        <v>18</v>
+      </c>
+      <c r="F23" s="6">
+        <v>18</v>
+      </c>
+      <c r="G23" s="6">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A24" t="s">
+        <v>28</v>
+      </c>
+      <c r="B24" s="6">
+        <v>29</v>
+      </c>
+      <c r="C24" s="6">
+        <v>29</v>
+      </c>
+      <c r="D24" s="6">
+        <v>29</v>
+      </c>
+      <c r="E24" s="6">
+        <v>29</v>
+      </c>
+      <c r="F24" s="6">
+        <v>29</v>
+      </c>
+      <c r="G24" s="6">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A25" t="s">
+        <v>29</v>
+      </c>
+      <c r="B25" s="6">
+        <v>11</v>
+      </c>
+      <c r="C25" s="6">
+        <v>11</v>
+      </c>
+      <c r="D25" s="6">
+        <v>11</v>
+      </c>
+      <c r="E25" s="6">
+        <v>11</v>
+      </c>
+      <c r="F25" s="6">
+        <v>11</v>
+      </c>
+      <c r="G25" s="6">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A26" t="s">
+        <v>30</v>
+      </c>
+      <c r="B26" s="6">
+        <v>1</v>
+      </c>
+      <c r="C26" s="6">
+        <v>1</v>
+      </c>
+      <c r="D26" s="6">
+        <v>1</v>
+      </c>
+      <c r="E26" s="6">
+        <v>1</v>
+      </c>
+      <c r="F26" s="6">
+        <v>1</v>
+      </c>
+      <c r="G26" s="6">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{772153BA-5CAE-46C1-BC4B-377C4E1B2C62}">
   <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A1" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>39</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="F2" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="F3" s="3" t="s">
         <v>51</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="D4" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="E4" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="F4" s="5" t="s">
         <v>57</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="F5" s="3" t="s">
         <v>63</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="D6" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="E6" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="F6" s="5" t="s">
         <v>69</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="D7" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="E7" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="F7" s="3" t="s">
         <v>75</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="D8" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="E8" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="F8" s="5" t="s">
         <v>81</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A9" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="E9" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="F9" s="3" t="s">
         <v>87</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A10" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="D10" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="E10" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="F10" s="5" t="s">
         <v>93</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A11" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="E11" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="F11" s="3" t="s">
         <v>99</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -1085,162 +1707,162 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85865546-6824-4C6D-A94B-4273F5B117D6}">
   <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>93</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" s="4" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B2" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>99</v>
-      </c>
       <c r="E2" s="5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" s="2" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>39</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A6" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C6" s="4" t="s">
+      <c r="D6" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>69</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A7" s="2" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>75</v>
-      </c>
       <c r="E7" s="3" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A8" s="4" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B8" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="E8" s="5" t="s">
         <v>81</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A9" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="E9" s="3" t="s">
         <v>86</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>88</v>
       </c>
     </row>
   </sheetData>
@@ -1248,107 +1870,107 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D798F37-0E69-419A-83C6-08D737C39BA3}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A1" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>81</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A2" s="4" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A3" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A4" s="4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A5" s="2" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A6" s="4" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B6" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>69</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A7" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D7" s="3" t="s">
         <v>73</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -1357,6 +1979,159 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9807935-B95D-4790-9FAE-DBBF51269EAF}">
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="3" max="3" width="16.06640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D1" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C2" t="s">
+        <v>112</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>109</v>
+      </c>
+      <c r="C3" t="s">
+        <v>113</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A5">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A6">
+        <v>2</v>
+      </c>
+      <c r="B6" t="s">
+        <v>110</v>
+      </c>
+      <c r="C6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A7">
+        <v>2</v>
+      </c>
+      <c r="B7" t="s">
+        <v>110</v>
+      </c>
+      <c r="C7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A8">
+        <v>2</v>
+      </c>
+      <c r="B8" t="s">
+        <v>110</v>
+      </c>
+      <c r="C8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A9">
+        <v>2</v>
+      </c>
+      <c r="B9" t="s">
+        <v>110</v>
+      </c>
+      <c r="C9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A10">
+        <v>2</v>
+      </c>
+      <c r="B10" t="s">
+        <v>110</v>
+      </c>
+      <c r="C10" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2465ECB-C836-4264-867A-034B6DF3E176}">
   <dimension ref="A1:A26"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1366,7 +2141,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.45">
@@ -1421,77 +2196,77 @@
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>18</v>
+        <v>112</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>23</v>
+        <v>113</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -1499,7 +2274,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA3D358C-A238-4518-9516-78D5730C6DCB}">
   <dimension ref="A1:G26"/>
   <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1760,7 +2535,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>18</v>
+        <v>112</v>
       </c>
       <c r="B12" s="6">
         <v>20</v>
@@ -1783,7 +2558,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B13" s="6">
         <v>6</v>
@@ -1806,7 +2581,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B14" s="6">
         <v>0</v>
@@ -1829,7 +2604,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B15" s="6">
         <v>25</v>
@@ -1852,7 +2627,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B16" s="6">
         <v>0</v>
@@ -1875,7 +2650,7 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>23</v>
+        <v>113</v>
       </c>
       <c r="B17" s="6">
         <v>0</v>
@@ -1898,7 +2673,7 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B18" s="6">
         <v>11</v>
@@ -1921,7 +2696,7 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B19" s="6">
         <v>21</v>
@@ -1944,7 +2719,7 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B20" s="6">
         <v>27</v>
@@ -1967,7 +2742,7 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B21" s="6">
         <v>16</v>
@@ -1990,7 +2765,7 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B22" s="6">
         <v>8</v>
@@ -2013,7 +2788,7 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B23" s="6">
         <v>0</v>
@@ -2036,7 +2811,7 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B24" s="6">
         <v>1</v>
@@ -2059,7 +2834,7 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B25" s="6">
         <v>10</v>
@@ -2082,7 +2857,7 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B26" s="6">
         <v>19</v>
@@ -2109,7 +2884,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B46B4ED8-D1CC-446D-B631-CA4BD3C11BB8}">
   <dimension ref="A1:G26"/>
   <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -2120,7 +2895,7 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.45">
       <c r="B1" s="6" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>3</v>
@@ -2370,7 +3145,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>18</v>
+        <v>112</v>
       </c>
       <c r="B12" s="6">
         <v>18</v>
@@ -2393,7 +3168,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B13" s="6">
         <v>29</v>
@@ -2416,7 +3191,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B14" s="6">
         <v>4</v>
@@ -2439,7 +3214,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B15" s="6">
         <v>17</v>
@@ -2462,7 +3237,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B16" s="6">
         <v>11</v>
@@ -2485,7 +3260,7 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>23</v>
+        <v>113</v>
       </c>
       <c r="B17" s="6">
         <v>5</v>
@@ -2508,7 +3283,7 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B18" s="6">
         <v>0</v>
@@ -2531,7 +3306,7 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B19" s="6">
         <v>0</v>
@@ -2554,7 +3329,7 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B20" s="6">
         <v>1</v>
@@ -2577,7 +3352,7 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B21" s="6">
         <v>12</v>
@@ -2600,7 +3375,7 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B22" s="6">
         <v>0</v>
@@ -2623,7 +3398,7 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B23" s="6">
         <v>16</v>
@@ -2646,7 +3421,7 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B24" s="6">
         <v>0</v>
@@ -2669,7 +3444,7 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B25" s="6">
         <v>27</v>
@@ -2692,7 +3467,7 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B26" s="6">
         <v>23</v>
@@ -2718,7 +3493,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C029223F-6758-4902-9C5F-9E64D02D7E32}">
   <dimension ref="A1:G26"/>
   <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -2732,7 +3507,7 @@
         <v>5</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>2</v>
@@ -2979,7 +3754,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>18</v>
+        <v>112</v>
       </c>
       <c r="B12" s="6">
         <v>9</v>
@@ -3002,7 +3777,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B13" s="6">
         <v>14</v>
@@ -3025,7 +3800,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B14" s="6">
         <v>6</v>
@@ -3048,7 +3823,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B15" s="6">
         <v>13</v>
@@ -3071,7 +3846,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B16" s="6">
         <v>17</v>
@@ -3094,7 +3869,7 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>23</v>
+        <v>113</v>
       </c>
       <c r="B17" s="6">
         <v>0</v>
@@ -3117,7 +3892,7 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B18" s="6">
         <v>5</v>
@@ -3140,7 +3915,7 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B19" s="6">
         <v>4</v>
@@ -3163,7 +3938,7 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B20" s="6">
         <v>3</v>
@@ -3186,7 +3961,7 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B21" s="6">
         <v>19</v>
@@ -3209,7 +3984,7 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B22" s="6">
         <v>0</v>
@@ -3232,7 +4007,7 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B23" s="6">
         <v>11</v>
@@ -3255,7 +4030,7 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B24" s="6">
         <v>12</v>
@@ -3278,7 +4053,7 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B25" s="6">
         <v>23</v>
@@ -3301,7 +4076,7 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B26" s="6">
         <v>20</v>
@@ -3327,7 +4102,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{239CD3BE-5976-4BD9-BE18-D390C4007798}">
   <dimension ref="A1:G26"/>
   <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -3344,7 +4119,7 @@
         <v>3</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E1" s="6" t="s">
         <v>6</v>
@@ -3588,7 +4363,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>18</v>
+        <v>112</v>
       </c>
       <c r="B12" s="6">
         <v>23</v>
@@ -3611,7 +4386,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B13" s="6">
         <v>13</v>
@@ -3634,7 +4409,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B14" s="6">
         <v>22</v>
@@ -3657,7 +4432,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B15" s="6">
         <v>3</v>
@@ -3680,7 +4455,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B16" s="6">
         <v>0</v>
@@ -3703,7 +4478,7 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>23</v>
+        <v>113</v>
       </c>
       <c r="B17" s="6">
         <v>21</v>
@@ -3726,7 +4501,7 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B18" s="6">
         <v>5</v>
@@ -3749,7 +4524,7 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B19" s="6">
         <v>0</v>
@@ -3772,7 +4547,7 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B20" s="6">
         <v>6</v>
@@ -3795,7 +4570,7 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B21" s="6">
         <v>24</v>
@@ -3818,7 +4593,7 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B22" s="6">
         <v>0</v>
@@ -3841,7 +4616,7 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B23" s="6">
         <v>2</v>
@@ -3864,7 +4639,7 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B24" s="6">
         <v>0</v>
@@ -3887,7 +4662,7 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B25" s="6">
         <v>20</v>
@@ -3910,7 +4685,7 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B26" s="6">
         <v>17</v>
@@ -3936,7 +4711,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB95A337-BA4E-432A-98B3-C98423D056BF}">
   <dimension ref="A1:G26"/>
   <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -3956,7 +4731,7 @@
         <v>2</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F1" s="6" t="s">
         <v>7</v>
@@ -4197,7 +4972,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>18</v>
+        <v>112</v>
       </c>
       <c r="B12" s="6">
         <v>12</v>
@@ -4220,7 +4995,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B13" s="6">
         <v>16</v>
@@ -4243,7 +5018,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B14" s="6">
         <v>11</v>
@@ -4266,7 +5041,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B15" s="6">
         <v>22</v>
@@ -4289,7 +5064,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B16" s="6">
         <v>0</v>
@@ -4312,7 +5087,7 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>23</v>
+        <v>113</v>
       </c>
       <c r="B17" s="6">
         <v>0</v>
@@ -4335,7 +5110,7 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B18" s="6">
         <v>29</v>
@@ -4358,7 +5133,7 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B19" s="6">
         <v>28</v>
@@ -4381,7 +5156,7 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B20" s="6">
         <v>27</v>
@@ -4404,7 +5179,7 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B21" s="6">
         <v>25</v>
@@ -4427,7 +5202,7 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B22" s="6">
         <v>4</v>
@@ -4450,7 +5225,7 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B23" s="6">
         <v>0</v>
@@ -4473,7 +5248,7 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B24" s="6">
         <v>0</v>
@@ -4496,7 +5271,7 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B25" s="6">
         <v>26</v>
@@ -4519,7 +5294,7 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B26" s="6">
         <v>21</v>
@@ -4545,7 +5320,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A889525-5E13-4FF1-B848-79F3031DC422}">
   <dimension ref="A1:G26"/>
   <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -4568,7 +5343,7 @@
         <v>6</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="G1" s="6" t="s">
         <v>4</v>
@@ -4806,7 +5581,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>18</v>
+        <v>112</v>
       </c>
       <c r="B12" s="6">
         <v>20</v>
@@ -4829,7 +5604,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B13" s="6">
         <v>16</v>
@@ -4852,7 +5627,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B14" s="6">
         <v>12</v>
@@ -4875,7 +5650,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B15" s="6">
         <v>26</v>
@@ -4898,7 +5673,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B16" s="6">
         <v>19</v>
@@ -4921,7 +5696,7 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>23</v>
+        <v>113</v>
       </c>
       <c r="B17" s="6">
         <v>0</v>
@@ -4944,7 +5719,7 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B18" s="6">
         <v>23</v>
@@ -4967,7 +5742,7 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B19" s="6">
         <v>15</v>
@@ -4990,7 +5765,7 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B20" s="6">
         <v>6</v>
@@ -5013,7 +5788,7 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B21" s="6">
         <v>13</v>
@@ -5036,7 +5811,7 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B22" s="6">
         <v>14</v>
@@ -5059,7 +5834,7 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B23" s="6">
         <v>27</v>
@@ -5082,7 +5857,7 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B24" s="6">
         <v>0</v>
@@ -5105,7 +5880,7 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B25" s="6">
         <v>0</v>
@@ -5128,7 +5903,7 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B26" s="6">
         <v>7</v>
@@ -5147,615 +5922,6 @@
       </c>
       <c r="G26" s="6">
         <v>7</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4F6C5ED-CE4B-4A90-947D-21DA231DC860}">
-  <dimension ref="A1:G26"/>
-  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <cols>
-    <col min="1" max="1" width="19.73046875" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="16384" width="9.1328125" style="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="B1" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="G1" s="6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="6">
-        <v>13</v>
-      </c>
-      <c r="C2" s="6">
-        <v>13</v>
-      </c>
-      <c r="D2" s="6">
-        <v>13</v>
-      </c>
-      <c r="E2" s="6">
-        <v>13</v>
-      </c>
-      <c r="F2" s="6">
-        <v>13</v>
-      </c>
-      <c r="G2" s="6">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="6">
-        <v>16</v>
-      </c>
-      <c r="C3" s="6">
-        <v>16</v>
-      </c>
-      <c r="D3" s="6">
-        <v>16</v>
-      </c>
-      <c r="E3" s="6">
-        <v>16</v>
-      </c>
-      <c r="F3" s="6">
-        <v>16</v>
-      </c>
-      <c r="G3" s="6">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="6">
-        <v>12</v>
-      </c>
-      <c r="C4" s="6">
-        <v>12</v>
-      </c>
-      <c r="D4" s="6">
-        <v>12</v>
-      </c>
-      <c r="E4" s="6">
-        <v>12</v>
-      </c>
-      <c r="F4" s="6">
-        <v>12</v>
-      </c>
-      <c r="G4" s="6">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="6">
-        <v>8</v>
-      </c>
-      <c r="C5" s="6">
-        <v>8</v>
-      </c>
-      <c r="D5" s="6">
-        <v>8</v>
-      </c>
-      <c r="E5" s="6">
-        <v>8</v>
-      </c>
-      <c r="F5" s="6">
-        <v>8</v>
-      </c>
-      <c r="G5" s="6">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="6">
-        <v>5</v>
-      </c>
-      <c r="C6" s="6">
-        <v>5</v>
-      </c>
-      <c r="D6" s="6">
-        <v>5</v>
-      </c>
-      <c r="E6" s="6">
-        <v>5</v>
-      </c>
-      <c r="F6" s="6">
-        <v>5</v>
-      </c>
-      <c r="G6" s="6">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" s="6">
-        <v>2</v>
-      </c>
-      <c r="C7" s="6">
-        <v>2</v>
-      </c>
-      <c r="D7" s="6">
-        <v>2</v>
-      </c>
-      <c r="E7" s="6">
-        <v>2</v>
-      </c>
-      <c r="F7" s="6">
-        <v>2</v>
-      </c>
-      <c r="G7" s="6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" s="6">
-        <v>3</v>
-      </c>
-      <c r="C8" s="6">
-        <v>3</v>
-      </c>
-      <c r="D8" s="6">
-        <v>3</v>
-      </c>
-      <c r="E8" s="6">
-        <v>3</v>
-      </c>
-      <c r="F8" s="6">
-        <v>3</v>
-      </c>
-      <c r="G8" s="6">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A9" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" s="6">
-        <v>9</v>
-      </c>
-      <c r="C9" s="6">
-        <v>9</v>
-      </c>
-      <c r="D9" s="6">
-        <v>9</v>
-      </c>
-      <c r="E9" s="6">
-        <v>9</v>
-      </c>
-      <c r="F9" s="6">
-        <v>9</v>
-      </c>
-      <c r="G9" s="6">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="6">
-        <v>27</v>
-      </c>
-      <c r="C10" s="6">
-        <v>27</v>
-      </c>
-      <c r="D10" s="6">
-        <v>27</v>
-      </c>
-      <c r="E10" s="6">
-        <v>27</v>
-      </c>
-      <c r="F10" s="6">
-        <v>27</v>
-      </c>
-      <c r="G10" s="6">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A11" t="s">
-        <v>17</v>
-      </c>
-      <c r="B11" s="6">
-        <v>17</v>
-      </c>
-      <c r="C11" s="6">
-        <v>17</v>
-      </c>
-      <c r="D11" s="6">
-        <v>17</v>
-      </c>
-      <c r="E11" s="6">
-        <v>17</v>
-      </c>
-      <c r="F11" s="6">
-        <v>17</v>
-      </c>
-      <c r="G11" s="6">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A12" t="s">
-        <v>18</v>
-      </c>
-      <c r="B12" s="6">
-        <v>23</v>
-      </c>
-      <c r="C12" s="6">
-        <v>23</v>
-      </c>
-      <c r="D12" s="6">
-        <v>23</v>
-      </c>
-      <c r="E12" s="6">
-        <v>23</v>
-      </c>
-      <c r="F12" s="6">
-        <v>23</v>
-      </c>
-      <c r="G12" s="6">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A13" t="s">
-        <v>19</v>
-      </c>
-      <c r="B13" s="6">
-        <v>15</v>
-      </c>
-      <c r="C13" s="6">
-        <v>15</v>
-      </c>
-      <c r="D13" s="6">
-        <v>15</v>
-      </c>
-      <c r="E13" s="6">
-        <v>15</v>
-      </c>
-      <c r="F13" s="6">
-        <v>15</v>
-      </c>
-      <c r="G13" s="6">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A14" t="s">
-        <v>20</v>
-      </c>
-      <c r="B14" s="6">
-        <v>0</v>
-      </c>
-      <c r="C14" s="6">
-        <v>0</v>
-      </c>
-      <c r="D14" s="6">
-        <v>0</v>
-      </c>
-      <c r="E14" s="6">
-        <v>0</v>
-      </c>
-      <c r="F14" s="6">
-        <v>0</v>
-      </c>
-      <c r="G14" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A15" t="s">
-        <v>21</v>
-      </c>
-      <c r="B15" s="6">
-        <v>28</v>
-      </c>
-      <c r="C15" s="6">
-        <v>28</v>
-      </c>
-      <c r="D15" s="6">
-        <v>28</v>
-      </c>
-      <c r="E15" s="6">
-        <v>28</v>
-      </c>
-      <c r="F15" s="6">
-        <v>28</v>
-      </c>
-      <c r="G15" s="6">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A16" t="s">
-        <v>22</v>
-      </c>
-      <c r="B16" s="6">
-        <v>14</v>
-      </c>
-      <c r="C16" s="6">
-        <v>14</v>
-      </c>
-      <c r="D16" s="6">
-        <v>14</v>
-      </c>
-      <c r="E16" s="6">
-        <v>14</v>
-      </c>
-      <c r="F16" s="6">
-        <v>14</v>
-      </c>
-      <c r="G16" s="6">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A17" t="s">
-        <v>23</v>
-      </c>
-      <c r="B17" s="6">
-        <v>24</v>
-      </c>
-      <c r="C17" s="6">
-        <v>24</v>
-      </c>
-      <c r="D17" s="6">
-        <v>24</v>
-      </c>
-      <c r="E17" s="6">
-        <v>24</v>
-      </c>
-      <c r="F17" s="6">
-        <v>24</v>
-      </c>
-      <c r="G17" s="6">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A18" t="s">
-        <v>24</v>
-      </c>
-      <c r="B18" s="6">
-        <v>0</v>
-      </c>
-      <c r="C18" s="6">
-        <v>0</v>
-      </c>
-      <c r="D18" s="6">
-        <v>0</v>
-      </c>
-      <c r="E18" s="6">
-        <v>0</v>
-      </c>
-      <c r="F18" s="6">
-        <v>0</v>
-      </c>
-      <c r="G18" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A19" t="s">
-        <v>25</v>
-      </c>
-      <c r="B19" s="6">
-        <v>0</v>
-      </c>
-      <c r="C19" s="6">
-        <v>0</v>
-      </c>
-      <c r="D19" s="6">
-        <v>0</v>
-      </c>
-      <c r="E19" s="6">
-        <v>0</v>
-      </c>
-      <c r="F19" s="6">
-        <v>0</v>
-      </c>
-      <c r="G19" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A20" t="s">
-        <v>26</v>
-      </c>
-      <c r="B20" s="6">
-        <v>6</v>
-      </c>
-      <c r="C20" s="6">
-        <v>6</v>
-      </c>
-      <c r="D20" s="6">
-        <v>6</v>
-      </c>
-      <c r="E20" s="6">
-        <v>6</v>
-      </c>
-      <c r="F20" s="6">
-        <v>6</v>
-      </c>
-      <c r="G20" s="6">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A21" t="s">
-        <v>27</v>
-      </c>
-      <c r="B21" s="6">
-        <v>19</v>
-      </c>
-      <c r="C21" s="6">
-        <v>19</v>
-      </c>
-      <c r="D21" s="6">
-        <v>19</v>
-      </c>
-      <c r="E21" s="6">
-        <v>19</v>
-      </c>
-      <c r="F21" s="6">
-        <v>19</v>
-      </c>
-      <c r="G21" s="6">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A22" t="s">
-        <v>28</v>
-      </c>
-      <c r="B22" s="6">
-        <v>25</v>
-      </c>
-      <c r="C22" s="6">
-        <v>25</v>
-      </c>
-      <c r="D22" s="6">
-        <v>25</v>
-      </c>
-      <c r="E22" s="6">
-        <v>25</v>
-      </c>
-      <c r="F22" s="6">
-        <v>25</v>
-      </c>
-      <c r="G22" s="6">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A23" t="s">
-        <v>29</v>
-      </c>
-      <c r="B23" s="6">
-        <v>18</v>
-      </c>
-      <c r="C23" s="6">
-        <v>18</v>
-      </c>
-      <c r="D23" s="6">
-        <v>18</v>
-      </c>
-      <c r="E23" s="6">
-        <v>18</v>
-      </c>
-      <c r="F23" s="6">
-        <v>18</v>
-      </c>
-      <c r="G23" s="6">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A24" t="s">
-        <v>30</v>
-      </c>
-      <c r="B24" s="6">
-        <v>29</v>
-      </c>
-      <c r="C24" s="6">
-        <v>29</v>
-      </c>
-      <c r="D24" s="6">
-        <v>29</v>
-      </c>
-      <c r="E24" s="6">
-        <v>29</v>
-      </c>
-      <c r="F24" s="6">
-        <v>29</v>
-      </c>
-      <c r="G24" s="6">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A25" t="s">
-        <v>31</v>
-      </c>
-      <c r="B25" s="6">
-        <v>11</v>
-      </c>
-      <c r="C25" s="6">
-        <v>11</v>
-      </c>
-      <c r="D25" s="6">
-        <v>11</v>
-      </c>
-      <c r="E25" s="6">
-        <v>11</v>
-      </c>
-      <c r="F25" s="6">
-        <v>11</v>
-      </c>
-      <c r="G25" s="6">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A26" t="s">
-        <v>32</v>
-      </c>
-      <c r="B26" s="6">
-        <v>1</v>
-      </c>
-      <c r="C26" s="6">
-        <v>1</v>
-      </c>
-      <c r="D26" s="6">
-        <v>1</v>
-      </c>
-      <c r="E26" s="6">
-        <v>1</v>
-      </c>
-      <c r="F26" s="6">
-        <v>1</v>
-      </c>
-      <c r="G26" s="6">
-        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>